<commit_message>
Last updates and analysis code
</commit_message>
<xml_diff>
--- a/n10-30-rundata.xlsx
+++ b/n10-30-rundata.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anter\Documents\Kursseja\Research_Training\Fluid-Drop_Optimizer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AF569E9-56FF-4F49-94A9-99C9C6B542AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFCAAB17-A1C7-4CDC-97BA-DF16C4DEC9FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="14592" xr2:uid="{D0E09B27-A212-46D0-A701-3BE87E223BED}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="14592" activeTab="1" xr2:uid="{D0E09B27-A212-46D0-A701-3BE87E223BED}"/>
   </bookViews>
   <sheets>
     <sheet name="time-dependence" sheetId="1" r:id="rId1"/>
-    <sheet name="errors" sheetId="6" r:id="rId2"/>
-    <sheet name="CPU-energy" sheetId="5" r:id="rId3"/>
-    <sheet name="CPU-volume" sheetId="4" r:id="rId4"/>
-    <sheet name="GPU-energy" sheetId="3" r:id="rId5"/>
-    <sheet name="GPU-volume" sheetId="2" r:id="rId6"/>
+    <sheet name="test comparisons" sheetId="7" r:id="rId2"/>
+    <sheet name="errors" sheetId="6" r:id="rId3"/>
+    <sheet name="CPU-energy" sheetId="5" r:id="rId4"/>
+    <sheet name="CPU-volume" sheetId="4" r:id="rId5"/>
+    <sheet name="GPU-energy" sheetId="3" r:id="rId6"/>
+    <sheet name="GPU-volume" sheetId="2" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="28">
   <si>
     <t>Minimizer</t>
   </si>
@@ -108,6 +108,27 @@
   </si>
   <si>
     <t>Normalized RMSE</t>
+  </si>
+  <si>
+    <t>Device: GPU</t>
+  </si>
+  <si>
+    <t>Grid: 20</t>
+  </si>
+  <si>
+    <t>Constraints</t>
+  </si>
+  <si>
+    <t>V + Boundary Points</t>
+  </si>
+  <si>
+    <t>V, BP and Modified contact line</t>
+  </si>
+  <si>
+    <t>Method: trust-constr</t>
+  </si>
+  <si>
+    <t>Diff in rel. to Inp.</t>
   </si>
 </sst>
 </file>
@@ -1660,6 +1681,206 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64A9E868-C0C1-4D0E-ABC5-E27C0B25B962}">
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="1" max="1" width="24.9453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.89453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.89453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.89453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.89453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.83984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.89453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3">
+        <v>3.6712934366865399E-6</v>
+      </c>
+      <c r="C4" s="3">
+        <v>3.5761716743322001E-6</v>
+      </c>
+      <c r="D4" s="3">
+        <v>3.9303744199148703E-6</v>
+      </c>
+      <c r="E4" s="3">
+        <f>((D4-$B4)/D4)*100</f>
+        <v>6.5917634186602996</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="3">
+        <v>3.6712934366865399E-6</v>
+      </c>
+      <c r="C5" s="3">
+        <v>3.5761716743322001E-6</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3.71598202722785E-6</v>
+      </c>
+      <c r="E5" s="3">
+        <f t="shared" ref="E5:E12" si="0">((D5-$B5)/D5)*100</f>
+        <v>1.2026051313990898</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="3">
+        <v>3.6712934366865399E-6</v>
+      </c>
+      <c r="C6" s="3">
+        <v>3.5761716743322001E-6</v>
+      </c>
+      <c r="D6" s="3">
+        <v>3.7139696030491299E-6</v>
+      </c>
+      <c r="E6" s="3">
+        <f t="shared" si="0"/>
+        <v>1.1490715036427148</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="E7" s="3"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="3">
+        <v>2.6829739468141001E-9</v>
+      </c>
+      <c r="C10" s="3">
+        <v>2.7254297745274302E-9</v>
+      </c>
+      <c r="D10" s="3">
+        <v>1.14271998524708E-8</v>
+      </c>
+      <c r="E10" s="3">
+        <f t="shared" si="0"/>
+        <v>76.521160201517048</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="3">
+        <v>2.6829739468141001E-9</v>
+      </c>
+      <c r="C11" s="3">
+        <v>2.7254297745274302E-9</v>
+      </c>
+      <c r="D11" s="3">
+        <v>2.6835486646545099E-9</v>
+      </c>
+      <c r="E11" s="3">
+        <f t="shared" si="0"/>
+        <v>2.1416337552564408E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="3">
+        <v>2.6829739468141001E-9</v>
+      </c>
+      <c r="C12" s="3">
+        <v>2.7254297745274302E-9</v>
+      </c>
+      <c r="D12" s="3">
+        <v>2.6835144135918002E-9</v>
+      </c>
+      <c r="E12" s="3">
+        <f t="shared" si="0"/>
+        <v>2.0140259912993851E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C28D7367-0449-4A3F-9C62-AAC83CA3629D}">
   <dimension ref="A1:M24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -2352,7 +2573,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A21B0054-6D26-48F5-91C4-8A5BC5D04F53}">
   <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -2954,7 +3175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A099A7F5-8017-4EC7-93FD-03A22C8B650F}">
   <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -3556,7 +3777,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A6583FE-60AC-4C96-A8C8-4A2335FD988F}">
   <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
@@ -4158,7 +4379,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7768C6E7-7A50-45F7-B18D-DA74A5E5CDB4}">
   <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>

</xml_diff>